<commit_message>
Add historical Ltd tax data (FY2020-FY2024) and HMRC reference documents
Tax data files created from HMRC published rates:
- app/data/ltd-2020.toml through ltd-2024.toml
- FY2020-2022: 19% flat CT rate (pre-two-tier)
- FY2023+: 19% small profits / 25% main rate with marginal relief
- Full expensing: 0% pre-FY2023, 100% from FY2023
- Employer NI: 13.8% pre-FY2025, 15% from FY2025
- Dividend tax: allowance reduced 2000 -> 1000 -> 500 over the period

HMRC reference documents downloaded:
- NI rates and earnings limits 2020-21 PDF
- NI contribution tables CA38 (Jul 2022, Jan-Apr 2024)
- NI contributions rates and allowances table (ODS)
- Capital allowances toolkit 2020 PDF

7 Ltd packages generated (FY2020-FY2026, Mar21 through Mar27).
120 tests passing.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages-generated/GB Accounts Company 2027-03-31 (Mar27) Excel 2007/Vatreturns.xlsx
+++ b/packages-generated/GB Accounts Company 2027-03-31 (Mar27) Excel 2007/Vatreturns.xlsx
@@ -40,7 +40,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="3">VATQtr4!$A$1:$I$31</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">VATQtr5!$A$1:$I$31</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="F5" s="126"/>
       <c r="G5" s="42">
-        <v>45838</v>
+        <v>46203</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="13"/>
@@ -13932,7 +13932,7 @@
       </c>
       <c r="F5" s="126"/>
       <c r="G5" s="42">
-        <v>45930</v>
+        <v>46295</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="13"/>
@@ -14498,7 +14498,7 @@
       </c>
       <c r="F5" s="126"/>
       <c r="G5" s="42">
-        <v>46022</v>
+        <v>46387</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="13"/>
@@ -15064,7 +15064,7 @@
       </c>
       <c r="F5" s="126"/>
       <c r="G5" s="42">
-        <v>46112</v>
+        <v>46477</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="13"/>
@@ -15630,7 +15630,7 @@
       </c>
       <c r="F5" s="126"/>
       <c r="G5" s="42">
-        <v>46142</v>
+        <v>46507</v>
       </c>
       <c r="H5" s="10"/>
       <c r="I5" s="13"/>

</xml_diff>